<commit_message>
Diss: February Data Processing and Collection Script Complete
</commit_message>
<xml_diff>
--- a/02_literature/00_reference_tracker.xlsx
+++ b/02_literature/00_reference_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/29cb6aa242dd6fa3/00_Documents/06_university/00_university_of_sussex/05_summer_semester/05_dissertation/02_literature/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{7D61B554-5378-4220-A798-A1246F7F0748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F50C88E-5C7F-4F8F-969E-E97F2B9BDF5C}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="8_{7D61B554-5378-4220-A798-A1246F7F0748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE6893C0-0946-480D-879D-CAC33184435E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{048EC744-F0B0-44F0-8D26-913D0BE8AFE5}"/>
+    <workbookView xWindow="34920" yWindow="2430" windowWidth="22065" windowHeight="11535" xr2:uid="{048EC744-F0B0-44F0-8D26-913D0BE8AFE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
   <si>
     <t xml:space="preserve">Paper </t>
   </si>
   <si>
-    <t>Summary</t>
-  </si>
-  <si>
     <t>Reference</t>
   </si>
   <si>
@@ -65,17 +62,185 @@
     <t>Overall</t>
   </si>
   <si>
-    <t>Specifc EU DSA TD Papers</t>
-  </si>
-  <si>
     <t>Content Moderation Paper</t>
+  </si>
+  <si>
+    <t>Published</t>
+  </si>
+  <si>
+    <t>Limitations</t>
+  </si>
+  <si>
+    <t>Automated Transparency: A Legal and Empirical Analysis of the DSA TD</t>
+  </si>
+  <si>
+    <t>Paper Aim</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>NL</t>
+  </si>
+  <si>
+    <t>Aim is to understand whether the TD helps the DSA live up to its transparency promises. To what extent the SOR design reflects conditions in Art 17. What are the compliance issues of moderation practices.</t>
+  </si>
+  <si>
+    <t>Data Used</t>
+  </si>
+  <si>
+    <t>All pltforms: google shopping, amazon, social media and google maps, booking.com - they also consider free text fields. Consider a ten day window between 19 and 23 November 2023.</t>
+  </si>
+  <si>
+    <t>1) Absolute figure of reports per company. Expectation that SOR numbers would be proportional to user number - not the case. 2) Level of automation in decision making - X, LinkedIn and Booking.com do not use any automation. Tiktok - automation for most SoRs. Correlation between automated detection and decision. 3) What percentage of all decisions are being declared as illegal content. X tops the social media companies here. Null values in decision_ground_reference_url. 4) What actions are being taken - content visibility restricted/account restrictions etc. 5) How  many times is content language populated - in roughly 50% of their sample. 6) Moderation delay - delay between content upload and action. Upload delay - delay between action and reporting.</t>
+  </si>
+  <si>
+    <t>Small sample of only 10 days and very wide scope of companies. Didn’t have data to really look into moderation delay - from their perspective it seems a bad thing if there is a large average between content upload and action date. However, it can be the case that it is a positive action for them to find a lot of historic content using automated means. X, for example, finds next to no historic content as everything is manual.</t>
+  </si>
+  <si>
+    <t>Discussion Points</t>
+  </si>
+  <si>
+    <t>1) Data is submitted by platforms themselves - so we can only look at what they tell us. 2) Illegal content is not being properly defined and most violations are noted as 'terms and conditions' violations. 3) Attempts to get more information by DSA in free field columns are being worked around by platforms - so this is not in the spirit of the legislation.</t>
+  </si>
+  <si>
+    <t>Rishabh Kaushal, Jacob Van De Kerkhof, Catalina Goanta, Gerasimos Spanakis, and Adriana Iamnitchi. 2024. Automated Transparency: A Legal and Empirical Analysis of the Digital Services Act Transparency Database. In Proceedings of the 2024 ACM Conference on Fairness, Accountability, and Transparency (FAccT '24). Association for Computing Machinery, New York, NY, USA, 1121–1132. https://doi.org/10.1145/3630106.3658960</t>
+  </si>
+  <si>
+    <t>One Day in Content Moderation: Analyzing 24 h of Social Media Platforms' Content Decisions through the DSA TD</t>
+  </si>
+  <si>
+    <t>Specifc EU DSA TD Paper</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>Dergacheva, D., Kuznetsova, V., Scharlach, R., &amp; Katzenbach, C. (2023): One Day in Content Moderation: Analyzing 24h of Social Media Platforms’ Content Decisions through the DSA Transparency Database. Lab Platform Governance, Media, and Technology (PGMT). Centre for Media, Communication and Information Research (ZeMKI), University of Bremen.</t>
+  </si>
+  <si>
+    <t>Facebook, Instagram, Tiktok, Youtube, X, Snapchat, Pinterest and LinkedIn - for one day - November 5th 2023 - 7.1 million decisions.</t>
+  </si>
+  <si>
+    <t>Interesting Points</t>
+  </si>
+  <si>
+    <t>Looks at whether decisions were automated or manual, visibility measures applied, which content categories were most subject to moderation.</t>
+  </si>
+  <si>
+    <t>Can get number of active monthly users in EU per millions. Motivation for not looking at Pinterest: data includes russia and turkey users.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculates moderation values per user. Distribution of automated and non-automated detection and decisions. Decision visibility per platform. Looks at some qualitative statements in the decision visibility free field. Type of content moderated (text, video, synthetic media). Number of SORs per high level category (animal welfare etc.). What moderation practices are more common for certain categories - content category and visibility decisions are correlated with X-squared tests. </t>
+  </si>
+  <si>
+    <t>High level overview - looking at only one day in high level aggregations</t>
+  </si>
+  <si>
+    <t>Need for longitudinal studies. Point out that limitation in detail on EU webiste (but I imagine this has been fixed with the powerBI report that they now have)</t>
+  </si>
+  <si>
+    <t>Content Moderation on Social Media in the EU: Insights From the DSA Transparency Database</t>
+  </si>
+  <si>
+    <t>Early look at content moderation performance of 156 million decisions. Aims: how frequently is social media content subject to moderation, how odten are different types of content moderated, what are specific reasons, extent of automation and actions. Regression analysis to estimate how the likelihood of automation of content moderation decisions varies across content types and legal grounds.</t>
+  </si>
+  <si>
+    <t>Collected all SORs for the first two months from September 25 2023. 156 million SORs.</t>
+  </si>
+  <si>
+    <t>LinkedIn - numbers of SORs here very small. Number of synthetic media is very small - around 3.8% (text in the report is incorrect)</t>
+  </si>
+  <si>
+    <t>They often look at the high level category reason for why content is removed. I wonder how many mix the quantitative and qualitative aspects of the data to get more insight. They look at simply 'cat_spec' I think. Only two months of data taken into account.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Differences in frequency - Tiktok performs 350 tims more moderation that X per user. Content type - test and videos more likely to be moderated. Primary reasons - falling outside scope of service - illegal/harmful speech and porongraphy. Not a lot of misinformation being moderated. Majority of content is detected and decided automatically except for X. Some platforms more likely to remove content, other reduce visibility. They can see the incompatible content/illegal content problem in the data - that majority of SORs declare incompatible content wheras X declares exclusively illegal content. Nice results for regression - they find that content is 32.143 times more likely to have an automated decision if it was detected automatically.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study implied differences and inconsistencies in content moderation practices of social media. Different platforms focus on different content. On X illegal/harmful speech and misinformation are rarely moderated. </t>
+  </si>
+  <si>
+    <t>Further Work Recomm</t>
+  </si>
+  <si>
+    <t>Longitudinal study needed</t>
+  </si>
+  <si>
+    <t>Longitudinal study needed. More research needed to understand how content removal or visibility reduction affect on-platform user behavior. Analysis of source content (not possible for me)</t>
+  </si>
+  <si>
+    <r>
+      <t>Drolsbach, C. P., &amp; Pröllochs, N. (2024, May). Content moderation on social media in the EU: Insights from the DSA Transparency Database. In </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="8"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Companion Proceedings of the ACM Web Conference 2024</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> (pp. 939-942).</t>
+    </r>
+  </si>
+  <si>
+    <t>The DSA Transparency Database: Auditing Self-Reported Moderation Actions by Social Media</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>353,12M records of social media platforms in the first 100 days of SOR platform.</t>
+  </si>
+  <si>
+    <t>Platform-wise comparative study of volume of moderation actions, grounds for decisions, types of applied restrictions, types of moderated content, timeliness in undertaking and submitting moderation actions and use of automation. Cross check of the contents of the database with the platform's own transparency reports.</t>
+  </si>
+  <si>
+    <t>Looking to see if the reports in SOR match the transparency reports - interesting to see for me too. A clear data limitation.</t>
+  </si>
+  <si>
+    <t>If transparency reports do or do not match what the companies are reporting elsewhere. This could be interesting. Also - they claim this is the first in-depth platform wise comparative analysis of moderation actions over an extended time period. But again - only 100 days.</t>
+  </si>
+  <si>
+    <t>1) Platforms adhere only in part to spirit and structure of database. 2) Database is inadequate. 3) Platform performance is very different in actions 4) database is inconsistent 5) platform X contains most inconsistencies.  Also took into account the number of monthly authenticated active recipients. Windsorized delays from content to application date performed. Shows actually quite a lot of older content being discovered for some platforms - 0 for X - they windsorized, of course, to reduce outliers in visualisations.</t>
+  </si>
+  <si>
+    <t>Complaints of how vague the information provided can be. Many complaints around what the columns actually mean - this is very valid - automated detection or decision does not tell us the extent to which it is automated.</t>
+  </si>
+  <si>
+    <t>Look at duration of restriction, territorial scope and free text decisions</t>
+  </si>
+  <si>
+    <t>Amaury Trujillo, Tiziano Fagni, and Stefano Cresci. 2025. The DSA Transparency Database: Auditing Self-reported Moderation Actions by Social Media. Proc. ACM Hum.-Comput. Interact. 9, 2, Article CSCW187 (May 2025), 28 pages. https://doi.org/10.1145/3711085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Search of Reason. Are Statements of Reason Under the Digital Services Act a Valuable Source of Information on Content Moderation Practices? </t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
+  <si>
+    <t>Eight social media companies for three-months July-September 2024</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,6 +256,25 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF333333"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -113,9 +297,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -454,56 +646,245 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58FDA32B-BAE2-4928-86F1-0CA76F681D21}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="255.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="36.88671875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="2" customWidth="1"/>
+    <col min="7" max="8" width="71" style="2" customWidth="1"/>
+    <col min="9" max="10" width="21.21875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="21" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="255.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>3</v>
+    <row r="1" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="L4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>2</v>
-      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="85.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="204.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>